<commit_message>
0.6.0: RI/SP coverage, existing commitments and Azure purchase recommendations
- cost/commitments.py: per-resource pricing model, reservation and savings plan
  utilization/expiry, Azure reservation and benefit recommendations (read-only)
- 01 report: RI/SP section, new Excel sheets, alternatives reported separately
- 02 report: note when recommended VMs are mostly covered by RI/SP
- Sample regenerated with invented RI/SP data; docs and version 0.6.0
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azs1\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-kk_29knp\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC252264-CC29-4709-B885-00D0045D9536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32655BD-CD7D-411F-B663-FC2D44C9880D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="3420" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-3645" yWindow="-13320" windowWidth="5970" windowHeight="10455" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="月度总览" sheetId="1" r:id="rId1"/>
@@ -27,36 +27,42 @@
     <sheet name="每日费用" sheetId="12" r:id="rId12"/>
     <sheet name="10月费用预测" sheetId="13" r:id="rId13"/>
     <sheet name="分摊与计价方式" sheetId="14" r:id="rId14"/>
-    <sheet name="建议与跟踪" sheetId="15" r:id="rId15"/>
-    <sheet name="数据库与缓存用量" sheetId="16" r:id="rId16"/>
-    <sheet name="存储容量与层级" sheetId="17" r:id="rId17"/>
-    <sheet name="日志摄取与保留" sheetId="18" r:id="rId18"/>
-    <sheet name="预算检查" sheetId="19" r:id="rId19"/>
-    <sheet name="数据覆盖与说明" sheetId="20" r:id="rId20"/>
+    <sheet name="RI与SP" sheetId="15" r:id="rId15"/>
+    <sheet name="Azure购买建议" sheetId="16" r:id="rId16"/>
+    <sheet name="建议与跟踪" sheetId="17" r:id="rId17"/>
+    <sheet name="数据库与缓存用量" sheetId="18" r:id="rId18"/>
+    <sheet name="存储容量与层级" sheetId="19" r:id="rId19"/>
+    <sheet name="日志摄取与保留" sheetId="20" r:id="rId20"/>
+    <sheet name="预算检查" sheetId="21" r:id="rId21"/>
+    <sheet name="数据覆盖与说明" sheetId="22" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'10月费用预测'!$A$3:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'9月资源费用'!$A$3:$F$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">Azure购买建议!$A$3:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">RI与SP!$A$3:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">业务组对比!$A$3:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">主要计量变化!$A$3:$K$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">分摊与计价方式!$A$3:$C$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">分摊与计价方式!$A$3:$C$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">区域对比!$A$3:$I$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">变化原因拆解!$A$3:$L$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">图表!$A$3:$J$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">增长与下降来源!$A$3:$H$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">存储容量与层级!$A$3:$M$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">建议与跟踪!$A$3:$L$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">数据库与缓存用量!$A$3:$M$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">数据覆盖与说明!$A$3:$B$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">日志摄取与保留!$A$3:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">存储容量与层级!$A$3:$M$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">建议与跟踪!$A$3:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">数据库与缓存用量!$A$3:$M$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">数据覆盖与说明!$A$3:$B$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">日志摄取与保留!$A$3:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">月度总览!$A$3:$C$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">服务对比!$A$3:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">每日费用!$A$3:$C$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">订阅对比!$A$3:$M$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">资源组对比!$A$3:$F$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">预算检查!$A$3:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">预算检查!$A$3:$I$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="12">'10月费用预测'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'9月资源费用'!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="15">Azure购买建议!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="14">RI与SP!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">业务组对比!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">主要计量变化!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="13">分摊与计价方式!$1:$3</definedName>
@@ -64,17 +70,17 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="6">变化原因拆解!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">图表!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">增长与下降来源!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="16">存储容量与层级!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="14">建议与跟踪!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="15">数据库与缓存用量!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="19">数据覆盖与说明!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="17">日志摄取与保留!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="18">存储容量与层级!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="16">建议与跟踪!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="17">数据库与缓存用量!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="21">数据覆盖与说明!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="19">日志摄取与保留!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">月度总览!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">服务对比!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">每日费用!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">订阅对比!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">资源组对比!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="18">预算检查!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="20">预算检查!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -94,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="571">
   <si>
     <t>示例客户：2026年9月成本巡检（对比8月）</t>
   </si>
@@ -168,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-27T02:32:52.730497+00:00</t>
+    <t>2026-10-27T06:11:07.154271+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -1143,15 +1149,144 @@
     <t>OnDemand</t>
   </si>
   <si>
+    <t>分摊费用/计价方式（按资源汇总）</t>
+  </si>
+  <si>
+    <t>ondemand</t>
+  </si>
+  <si>
+    <t>reservation</t>
+  </si>
+  <si>
+    <t>现有预留实例（RI）和节省计划（SP）</t>
+  </si>
+  <si>
+    <t>使用率来自 Azure；近 30 天低于 80% 视为未用满，90 天内到期单独提示。读不到订单时不代表没有购买。</t>
+  </si>
+  <si>
+    <t>名称</t>
+  </si>
+  <si>
+    <t>规格或承诺</t>
+  </si>
+  <si>
+    <t>范围</t>
+  </si>
+  <si>
+    <t>期限</t>
+  </si>
+  <si>
+    <t>近7天使用率%</t>
+  </si>
+  <si>
+    <t>近30天使用率%</t>
+  </si>
+  <si>
+    <t>到期日期</t>
+  </si>
+  <si>
+    <t>提示</t>
+  </si>
+  <si>
+    <t>预留实例</t>
+  </si>
+  <si>
+    <t>shop-web-d4sv5</t>
+  </si>
+  <si>
+    <t>Standard_D4s_v5</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>1 年</t>
+  </si>
+  <si>
+    <t>2027-03-31</t>
+  </si>
+  <si>
+    <t>正常</t>
+  </si>
+  <si>
+    <t>legacy-report-e16sv5</t>
+  </si>
+  <si>
+    <t>Standard_E16s_v5</t>
+  </si>
+  <si>
+    <t>Shared</t>
+  </si>
+  <si>
+    <t>2027-05-31</t>
+  </si>
+  <si>
+    <t>近 30 天使用率 0%，未用满</t>
+  </si>
+  <si>
+    <t>节省计划</t>
+  </si>
+  <si>
+    <t>compute-sp-2025</t>
+  </si>
+  <si>
+    <t>每小时承诺 USD 1.20</t>
+  </si>
+  <si>
+    <t>2026-12-15</t>
+  </si>
+  <si>
+    <t>49 天后到期，未设置自动续订</t>
+  </si>
+  <si>
+    <t>Azure 基于过去 30 天用量的 RI/SP 购买建议</t>
+  </si>
+  <si>
+    <t>金额为 Azure 估算的 30 天费用和节省（约等于每月），按当前用量计算，未考虑降配；先降配并稳定后再按新的用量采购。同一订阅的 1 年和 3 年、预留实例和节省计划是互相替代的方案，节省不能相加。</t>
+  </si>
+  <si>
+    <t>类型</t>
+  </si>
+  <si>
+    <t>资源类型</t>
+  </si>
+  <si>
+    <t>规格</t>
+  </si>
+  <si>
+    <t>建议数量或每小时承诺</t>
+  </si>
+  <si>
+    <t>30天按需费用USD</t>
+  </si>
+  <si>
+    <t>购买后费用USD</t>
+  </si>
+  <si>
+    <t>估算节省USD（30天）</t>
+  </si>
+  <si>
+    <t>VirtualMachines</t>
+  </si>
+  <si>
+    <t>japaneast</t>
+  </si>
+  <si>
+    <t>3 年</t>
+  </si>
+  <si>
+    <t>Compute_Savings_Plan</t>
+  </si>
+  <si>
+    <t>每小时承诺 0.95</t>
+  </si>
+  <si>
     <t>建议清单和执行跟踪</t>
   </si>
   <si>
     <t>预计节省不是已实现节省；当前检查建议与历史费用分别标注。</t>
   </si>
   <si>
-    <t>范围</t>
-  </si>
-  <si>
     <t>发现</t>
   </si>
   <si>
@@ -1257,7 +1392,7 @@
     <t>长期稳定计算、数据库、缓存及可预留存储费用</t>
   </si>
   <si>
-    <t>已有按服务列表价对比；是否有闲置承诺需结合现有订单及使用记录核对</t>
+    <t>9月分摊费用中 8.3% 由 RI/SP 覆盖；现有 2 个预留、1 个节省计划，其中 1 个近 30 天未用满，1 个即将到期；Azure 基于过去 30 天用量估算，购买 1 年期预留实例约节省 USD 128.62，购买 1 年期节省计划约节省 USD 188.60（每 30 天，按当前用量、未计入降配；预留实例和节省计划覆盖同一部分用量，只能选其一，3 年期方案见 Excel）</t>
   </si>
   <si>
     <t>先确定调整后的长期用量，再比较适用的1年/3年RI和SP；不要按全年满配估算直接采购</t>
@@ -1338,15 +1473,6 @@
     <t>按每日平均值计算9月加权平均。规格为10月26日的当前配置，不一定是9月配置。CPU和内存都低于20%只表示可做容量评审，不代表可以直接降配。</t>
   </si>
   <si>
-    <t>名称</t>
-  </si>
-  <si>
-    <t>类型</t>
-  </si>
-  <si>
-    <t>规格</t>
-  </si>
-  <si>
     <t>9月费用USD</t>
   </si>
   <si>
@@ -1380,9 +1506,6 @@
     <t>Standard_D4ds_v4</t>
   </si>
   <si>
-    <t>japaneast</t>
-  </si>
-  <si>
     <t>CPU和内存9月平均均低于20%，建议容量评审</t>
   </si>
   <si>
@@ -1627,6 +1750,24 @@
   </si>
   <si>
     <t>对5个有费用订阅查询预算：4个无预算记录，shop-prod有月度USD 15,000预算；其余1个订阅未查询预算。年度累计支出不作为9月超预算证明</t>
+  </si>
+  <si>
+    <t>RI/SP 覆盖（按资源）</t>
+  </si>
+  <si>
+    <t>4 个有费用的订阅读取成功（9月分摊费用，按资源和计价方式）</t>
+  </si>
+  <si>
+    <t>RI/SP 现有订单</t>
+  </si>
+  <si>
+    <t>预留：读取成功；节省计划：读取成功</t>
+  </si>
+  <si>
+    <t>Azure 购买建议</t>
+  </si>
+  <si>
+    <t>6/6 次查询成功，共 3 条建议</t>
   </si>
   <si>
     <t>按区域费用</t>
@@ -2158,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-74B2-42B4-9DA5-487FA8472E6D}"/>
+              <c16:uniqueId val="{00000000-B053-4822-A0CB-B1770A835C3E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2480,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-74B2-42B4-9DA5-487FA8472E6D}"/>
+              <c16:uniqueId val="{00000001-B053-4822-A0CB-B1770A835C3E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2778,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-110A-4306-A70F-3E27673AAEC3}"/>
+              <c16:uniqueId val="{00000000-753A-4C6B-8439-D87CB773F152}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2935,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-110A-4306-A70F-3E27673AAEC3}"/>
+              <c16:uniqueId val="{00000001-753A-4C6B-8439-D87CB773F152}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3170,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-110A-4306-A70F-3E27673AAEC3}"/>
+              <c16:uniqueId val="{00000002-753A-4C6B-8439-D87CB773F152}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3337,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D017-4DDE-96D5-91756C15346E}"/>
+              <c16:uniqueId val="{00000000-0F8D-48FF-908F-07C42B280513}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3425,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D017-4DDE-96D5-91756C15346E}"/>
+              <c16:uniqueId val="{00000001-0F8D-48FF-908F-07C42B280513}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3549,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{00000001-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3570,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{00000003-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3591,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{00000005-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3612,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{00000007-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3622,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{00000009-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3632,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{0000000B-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3642,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{0000000D-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3652,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{0000000F-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3662,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{00000011-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3672,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-1F2F-4813-B831-5CAB723525E7}"/>
+                <c16:uniqueId val="{00000013-7042-4AB8-A216-A2A24AE1475A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3755,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-1F2F-4813-B831-5CAB723525E7}"/>
+              <c16:uniqueId val="{00000014-7042-4AB8-A216-A2A24AE1475A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3875,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-7ADC-4746-B3D5-6F9AE7B46876}"/>
+                <c16:uniqueId val="{00000001-1F94-48D9-B4C9-8FE5828FB4FA}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-7ADC-4746-B3D5-6F9AE7B46876}"/>
+                <c16:uniqueId val="{00000003-1F94-48D9-B4C9-8FE5828FB4FA}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3931,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-7ADC-4746-B3D5-6F9AE7B46876}"/>
+              <c16:uniqueId val="{00000004-1F94-48D9-B4C9-8FE5828FB4FA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6247,7 +6388,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -6422,8 +6563,30 @@
         <v>17350.942500000001</v>
       </c>
     </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C17" s="12">
+        <v>2357.2800000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="C18" s="5">
+        <v>214.28</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:C16" xr:uid="{00000000-0009-0000-0000-00000D000000}"/>
+  <autoFilter ref="A3:C18" xr:uid="{00000000-0009-0000-0000-00000D000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -6435,6 +6598,342 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="9" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
+        <v>352</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+    </row>
+    <row r="2" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+    </row>
+    <row r="3" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F4" s="5">
+        <v>99</v>
+      </c>
+      <c r="G4" s="5">
+        <v>98.5</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="F5" s="12">
+        <v>0</v>
+      </c>
+      <c r="G5" s="12">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="25" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F6" s="5">
+        <v>99.6</v>
+      </c>
+      <c r="G6" s="5">
+        <v>99.2</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>378</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:I6" xr:uid="{00000000-0009-0000-0000-00000E000000}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="10" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
+        <v>379</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+    </row>
+    <row r="2" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+    </row>
+    <row r="3" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G4" s="5">
+        <v>2</v>
+      </c>
+      <c r="H4" s="5">
+        <v>357.12</v>
+      </c>
+      <c r="I4" s="5">
+        <v>228.5</v>
+      </c>
+      <c r="J4" s="5">
+        <v>128.62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="G5" s="12">
+        <v>2</v>
+      </c>
+      <c r="H5" s="12">
+        <v>357.12</v>
+      </c>
+      <c r="I5" s="12">
+        <v>146.4</v>
+      </c>
+      <c r="J5" s="12">
+        <v>210.72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G6" s="5">
+        <v>0.95</v>
+      </c>
+      <c r="H6" s="5">
+        <v>1062</v>
+      </c>
+      <c r="I6" s="5">
+        <v>873.4</v>
+      </c>
+      <c r="J6" s="5">
+        <v>188.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:J6" xr:uid="{00000000-0009-0000-0000-00000F000000}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -6449,7 +6948,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
-        <v>349</v>
+        <v>393</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -6465,7 +6964,7 @@
     </row>
     <row r="2" spans="1:12" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
-        <v>350</v>
+        <v>394</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
@@ -6484,61 +6983,61 @@
         <v>344</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>352</v>
+        <v>395</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>353</v>
+        <v>396</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>354</v>
+        <v>397</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>355</v>
+        <v>398</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>356</v>
+        <v>399</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>357</v>
+        <v>400</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>358</v>
+        <v>401</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>359</v>
+        <v>402</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>360</v>
+        <v>403</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>361</v>
+        <v>404</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>362</v>
+        <v>405</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>363</v>
+        <v>406</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>364</v>
+        <v>407</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>365</v>
+        <v>408</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4" t="s">
-        <v>366</v>
+        <v>409</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>367</v>
+        <v>410</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>368</v>
+        <v>411</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
@@ -6547,26 +7046,26 @@
     </row>
     <row r="5" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>362</v>
+        <v>405</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>369</v>
+        <v>412</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>370</v>
+        <v>413</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>371</v>
+        <v>414</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>366</v>
+        <v>409</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>367</v>
+        <v>410</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>368</v>
+        <v>411</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -6575,26 +7074,26 @@
     </row>
     <row r="6" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>362</v>
+        <v>405</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>372</v>
+        <v>415</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>373</v>
+        <v>416</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>374</v>
+        <v>417</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4" t="s">
-        <v>366</v>
+        <v>409</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>367</v>
+        <v>410</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>368</v>
+        <v>411</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
@@ -6603,26 +7102,26 @@
     </row>
     <row r="7" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>362</v>
+        <v>405</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>375</v>
+        <v>418</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>376</v>
+        <v>419</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>377</v>
+        <v>420</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>366</v>
+        <v>409</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>367</v>
+        <v>410</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>368</v>
+        <v>411</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -6631,28 +7130,28 @@
     </row>
     <row r="8" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>378</v>
+        <v>421</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>379</v>
+        <v>422</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>380</v>
+        <v>423</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>381</v>
+        <v>424</v>
       </c>
       <c r="E8" s="5">
         <v>760.51400000000001</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>382</v>
+        <v>425</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>383</v>
+        <v>426</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>384</v>
+        <v>427</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
@@ -6661,26 +7160,26 @@
     </row>
     <row r="9" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>385</v>
+        <v>428</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>386</v>
+        <v>429</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>387</v>
+        <v>430</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>388</v>
+        <v>431</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>389</v>
+        <v>432</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>390</v>
+        <v>433</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>391</v>
+        <v>434</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -6689,26 +7188,26 @@
     </row>
     <row r="10" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>392</v>
+        <v>435</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>393</v>
+        <v>436</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>394</v>
+        <v>437</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>395</v>
+        <v>438</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4" t="s">
-        <v>396</v>
+        <v>439</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>397</v>
+        <v>440</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>398</v>
+        <v>441</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -6717,26 +7216,26 @@
     </row>
     <row r="11" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>399</v>
+        <v>442</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>400</v>
+        <v>443</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>401</v>
+        <v>444</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>402</v>
+        <v>445</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>403</v>
+        <v>446</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>367</v>
+        <v>410</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>404</v>
+        <v>447</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -6745,26 +7244,26 @@
     </row>
     <row r="12" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>405</v>
+        <v>448</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>406</v>
+        <v>449</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>407</v>
+        <v>450</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>408</v>
+        <v>451</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4" t="s">
-        <v>409</v>
+        <v>452</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>410</v>
+        <v>453</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>411</v>
+        <v>454</v>
       </c>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
@@ -6772,7 +7271,7 @@
       <c r="L12" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L12" xr:uid="{00000000-0009-0000-0000-00000E000000}"/>
+  <autoFilter ref="A3:L12" xr:uid="{00000000-0009-0000-0000-000010000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
@@ -6782,8 +7281,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -6794,7 +7293,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
-        <v>412</v>
+        <v>455</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -6811,7 +7310,7 @@
     </row>
     <row r="2" spans="1:13" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
-        <v>413</v>
+        <v>456</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
@@ -6834,34 +7333,34 @@
         <v>244</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>414</v>
+        <v>354</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>415</v>
+        <v>381</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>416</v>
+        <v>383</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>150</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>417</v>
+        <v>457</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>418</v>
+        <v>458</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>419</v>
+        <v>459</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>420</v>
+        <v>460</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>421</v>
+        <v>461</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>422</v>
+        <v>462</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>4</v>
@@ -6878,13 +7377,13 @@
         <v>260</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>423</v>
+        <v>463</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>424</v>
+        <v>464</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>425</v>
+        <v>465</v>
       </c>
       <c r="G4" s="5">
         <v>1245</v>
@@ -6915,13 +7414,13 @@
         <v>266</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>426</v>
+        <v>466</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>427</v>
+        <v>467</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>428</v>
+        <v>389</v>
       </c>
       <c r="G5" s="12">
         <v>708</v>
@@ -6940,7 +7439,7 @@
         <v>30</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>429</v>
+        <v>468</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
@@ -6954,13 +7453,13 @@
         <v>264</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>426</v>
+        <v>466</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>427</v>
+        <v>467</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>428</v>
+        <v>389</v>
       </c>
       <c r="G6" s="5">
         <v>708</v>
@@ -6991,13 +7490,13 @@
         <v>268</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>423</v>
+        <v>463</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>430</v>
+        <v>469</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>428</v>
+        <v>389</v>
       </c>
       <c r="G7" s="12">
         <v>572.70000000000005</v>
@@ -7016,7 +7515,7 @@
         <v>23</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>431</v>
+        <v>470</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="25" x14ac:dyDescent="0.35">
@@ -7030,13 +7529,13 @@
         <v>274</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>432</v>
+        <v>471</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>433</v>
+        <v>472</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>428</v>
+        <v>389</v>
       </c>
       <c r="G8" s="5">
         <v>396</v>
@@ -7055,7 +7554,7 @@
         <v>30</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>434</v>
+        <v>473</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
@@ -7069,13 +7568,13 @@
         <v>298</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>426</v>
+        <v>466</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>435</v>
+        <v>474</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>428</v>
+        <v>389</v>
       </c>
       <c r="G9" s="12">
         <v>123</v>
@@ -7094,11 +7593,11 @@
         <v>30</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>429</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M9" xr:uid="{00000000-0009-0000-0000-00000F000000}"/>
+  <autoFilter ref="A3:M9" xr:uid="{00000000-0009-0000-0000-000011000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
@@ -7108,8 +7607,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -7121,7 +7620,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
-        <v>436</v>
+        <v>475</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -7138,7 +7637,7 @@
     </row>
     <row r="2" spans="1:13" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
-        <v>437</v>
+        <v>476</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
@@ -7161,37 +7660,37 @@
         <v>244</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>438</v>
+        <v>477</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>439</v>
+        <v>478</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>440</v>
+        <v>479</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>441</v>
+        <v>480</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>442</v>
+        <v>481</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>443</v>
+        <v>482</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>444</v>
+        <v>483</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>445</v>
+        <v>484</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>446</v>
+        <v>485</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>447</v>
+        <v>486</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>417</v>
+        <v>457</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
@@ -7205,10 +7704,10 @@
         <v>270</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>448</v>
+        <v>487</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>449</v>
+        <v>488</v>
       </c>
       <c r="F4" s="5">
         <v>22340</v>
@@ -7223,13 +7722,13 @@
         <v>18.170000000000002</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>450</v>
+        <v>489</v>
       </c>
       <c r="K4" s="5">
         <v>310</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>451</v>
+        <v>490</v>
       </c>
       <c r="M4" s="5">
         <v>477.65</v>
@@ -7246,10 +7745,10 @@
         <v>300</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>448</v>
+        <v>487</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>449</v>
+        <v>488</v>
       </c>
       <c r="F5" s="12">
         <v>4750</v>
@@ -7264,13 +7763,13 @@
         <v>10.95</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>452</v>
+        <v>491</v>
       </c>
       <c r="K5" s="12">
         <v>2400</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>453</v>
+        <v>492</v>
       </c>
       <c r="M5" s="12">
         <v>98.37</v>
@@ -7287,10 +7786,10 @@
         <v>326</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>448</v>
+        <v>487</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>449</v>
+        <v>488</v>
       </c>
       <c r="F6" s="5">
         <v>662</v>
@@ -7305,250 +7804,23 @@
         <v>8.76</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>454</v>
+        <v>493</v>
       </c>
       <c r="K6" s="5">
         <v>12</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>451</v>
+        <v>490</v>
       </c>
       <c r="M6" s="5">
         <v>13.54</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M6" xr:uid="{00000000-0009-0000-0000-000010000000}"/>
+  <autoFilter ref="A3:M6" xr:uid="{00000000-0009-0000-0000-000012000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="80" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="17" t="s">
-        <v>455</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-    </row>
-    <row r="2" spans="1:8" ht="52" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="18" t="s">
-        <v>456</v>
-      </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-    </row>
-    <row r="3" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="C4" s="5">
-        <v>3556.31</v>
-      </c>
-      <c r="D4" s="5">
-        <v>1290</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="F4" s="5">
-        <v>30</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>464</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="C5" s="12">
-        <v>1815.53</v>
-      </c>
-      <c r="D5" s="12">
-        <v>560</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="F5" s="12">
-        <v>30</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>467</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:H5" xr:uid="{00000000-0009-0000-0000-000011000000}"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="9" width="24" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="17" t="s">
-        <v>468</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-    </row>
-    <row r="2" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="18" t="s">
-        <v>469</v>
-      </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-    </row>
-    <row r="3" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>470</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>472</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>473</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>476</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="C4" s="5">
-        <v>15000</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>478</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>479</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>480</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>481</v>
-      </c>
-      <c r="H4" s="5">
-        <v>11840</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>482</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:I4" xr:uid="{00000000-0009-0000-0000-000012000000}"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
@@ -9190,7 +9462,234 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
+        <v>494</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+    </row>
+    <row r="2" spans="1:8" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="18" t="s">
+        <v>495</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+    </row>
+    <row r="3" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="25" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C4" s="5">
+        <v>3556.31</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1290</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="F4" s="5">
+        <v>30</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="25" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C5" s="12">
+        <v>1815.53</v>
+      </c>
+      <c r="D5" s="12">
+        <v>560</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="F5" s="12">
+        <v>30</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>506</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:H5" xr:uid="{00000000-0009-0000-0000-000013000000}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="9" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+    </row>
+    <row r="2" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="18" t="s">
+        <v>508</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+    </row>
+    <row r="3" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="C4" s="5">
+        <v>15000</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="H4" s="5">
+        <v>11840</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>521</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:I4" xr:uid="{00000000-0009-0000-0000-000014000000}"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -9199,13 +9698,13 @@
   <sheetData>
     <row r="1" spans="1:2" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
-        <v>483</v>
+        <v>522</v>
       </c>
       <c r="B1" s="17"/>
     </row>
     <row r="2" spans="1:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
-        <v>484</v>
+        <v>523</v>
       </c>
       <c r="B2" s="18"/>
     </row>
@@ -9219,26 +9718,26 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>485</v>
+        <v>524</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>486</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>487</v>
+        <v>526</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>486</v>
+        <v>525</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>488</v>
+        <v>527</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>486</v>
+        <v>525</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -9246,169 +9745,193 @@
         <v>250</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>486</v>
+        <v>525</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>489</v>
+        <v>528</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>490</v>
+        <v>529</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="25" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>491</v>
+        <v>530</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>492</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>493</v>
+        <v>532</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>494</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>495</v>
+        <v>534</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>496</v>
+        <v>535</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>497</v>
+        <v>536</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>498</v>
+        <v>537</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>499</v>
+        <v>538</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>500</v>
+        <v>539</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>501</v>
+        <v>540</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>502</v>
+        <v>541</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>503</v>
+        <v>542</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>504</v>
+        <v>543</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>505</v>
+        <v>544</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>506</v>
+        <v>545</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>507</v>
+        <v>546</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>508</v>
+        <v>547</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
-        <v>509</v>
+        <v>548</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>510</v>
+        <v>549</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>511</v>
+        <v>550</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="25" x14ac:dyDescent="0.35">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>513</v>
+        <v>552</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>514</v>
+        <v>553</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>515</v>
+        <v>554</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="25" x14ac:dyDescent="0.35">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>517</v>
+        <v>556</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="25" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>438</v>
+        <v>558</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="25" x14ac:dyDescent="0.35">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
-        <v>520</v>
+        <v>560</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="25" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>522</v>
+        <v>562</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>523</v>
+        <v>563</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
-        <v>524</v>
+        <v>477</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>525</v>
+        <v>564</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="25" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>570</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B26" xr:uid="{00000000-0009-0000-0000-000013000000}"/>
+  <autoFilter ref="A3:B29" xr:uid="{00000000-0009-0000-0000-000015000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B17" r:id="rId1" xr:uid="{00000000-0004-0000-1300-000000000000}"/>
+    <hyperlink ref="B17" r:id="rId1" xr:uid="{00000000-0004-0000-1500-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
0.6.1: fixes from a full GitHub Copilot run
- access-check reads the account's role assignments and warns about roles that can write
- 03 report: architecture overview (subscriptions, regions, main components, network) plus narrative 'architecture'
- 05 report: say so when the standard deployment tag or vendor rules were not provided; skip the business-line chart when no business lines are configured
- 00 report: correct the price-source sentence (actual bill vs public list price); neutral account wording
- Built-in Chinese names for common regions
- SKILL/writing rules: edit reports only through narrative files, state 'needs customer confirmation' once, name specific resources
- README: Copilot non-interactive run with an allow/deny tool list
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-kk_29knp\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-lhcbnfs4\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32655BD-CD7D-411F-B663-FC2D44C9880D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A50E3BD1-B771-45F7-BC59-1A52134C66E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3645" yWindow="-13320" windowWidth="5970" windowHeight="10455" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17190" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="月度总览" sheetId="1" r:id="rId1"/>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-27T06:11:07.154271+00:00</t>
+    <t>2026-10-27T09:26:35.021356+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B053-4822-A0CB-B1770A835C3E}"/>
+              <c16:uniqueId val="{00000000-CDAE-460F-BCCE-74A8137F1167}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B053-4822-A0CB-B1770A835C3E}"/>
+              <c16:uniqueId val="{00000001-CDAE-460F-BCCE-74A8137F1167}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-753A-4C6B-8439-D87CB773F152}"/>
+              <c16:uniqueId val="{00000000-5E10-4462-AC03-E5B9BBD2724D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-753A-4C6B-8439-D87CB773F152}"/>
+              <c16:uniqueId val="{00000001-5E10-4462-AC03-E5B9BBD2724D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-753A-4C6B-8439-D87CB773F152}"/>
+              <c16:uniqueId val="{00000002-5E10-4462-AC03-E5B9BBD2724D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0F8D-48FF-908F-07C42B280513}"/>
+              <c16:uniqueId val="{00000000-B06F-45F8-A1FD-43F7D72A1C92}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-0F8D-48FF-908F-07C42B280513}"/>
+              <c16:uniqueId val="{00000001-B06F-45F8-A1FD-43F7D72A1C92}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{00000001-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{00000003-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{00000005-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{00000007-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{00000009-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{0000000B-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{0000000D-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{0000000F-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{00000011-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-7042-4AB8-A216-A2A24AE1475A}"/>
+                <c16:uniqueId val="{00000013-DB4A-4C4C-991C-1B1B262B3EB3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-7042-4AB8-A216-A2A24AE1475A}"/>
+              <c16:uniqueId val="{00000014-DB4A-4C4C-991C-1B1B262B3EB3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-1F94-48D9-B4C9-8FE5828FB4FA}"/>
+                <c16:uniqueId val="{00000001-B1FA-42F5-84AC-FB2EB795E11C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-1F94-48D9-B4C9-8FE5828FB4FA}"/>
+                <c16:uniqueId val="{00000003-B1FA-42F5-84AC-FB2EB795E11C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-1F94-48D9-B4C9-8FE5828FB4FA}"/>
+              <c16:uniqueId val="{00000004-B1FA-42F5-84AC-FB2EB795E11C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
0.6.2: fixes found while rebuilding a real run offline
- Subscription Owner check: flag more than 3 owners (Microsoft's limit is 3), not 3 or more
- Each report clears its own old charts before drawing, so charts no longer produced do not linger
- 01: compare subscriptions instead of a single 'other' business group when no business lines are configured
- 03 architecture: plain wording when there are no VNet peerings
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-lhcbnfs4\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-yb_0tvu1\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A50E3BD1-B771-45F7-BC59-1A52134C66E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE7CB789-C94B-4F32-AEED-2718A9E86021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17190" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-27T09:26:35.021356+00:00</t>
+    <t>2026-10-27T09:56:53.145316+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-CDAE-460F-BCCE-74A8137F1167}"/>
+              <c16:uniqueId val="{00000000-2C6F-4FAE-9EB0-C59B49A42ADE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-CDAE-460F-BCCE-74A8137F1167}"/>
+              <c16:uniqueId val="{00000001-2C6F-4FAE-9EB0-C59B49A42ADE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5E10-4462-AC03-E5B9BBD2724D}"/>
+              <c16:uniqueId val="{00000000-C503-49C3-9E91-6C224CBF0505}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5E10-4462-AC03-E5B9BBD2724D}"/>
+              <c16:uniqueId val="{00000001-C503-49C3-9E91-6C224CBF0505}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-5E10-4462-AC03-E5B9BBD2724D}"/>
+              <c16:uniqueId val="{00000002-C503-49C3-9E91-6C224CBF0505}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B06F-45F8-A1FD-43F7D72A1C92}"/>
+              <c16:uniqueId val="{00000000-DA88-423D-BC40-4BE8BF19FCB0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B06F-45F8-A1FD-43F7D72A1C92}"/>
+              <c16:uniqueId val="{00000001-DA88-423D-BC40-4BE8BF19FCB0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{00000001-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{00000003-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{00000005-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{00000007-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{00000009-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{0000000B-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{0000000D-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{0000000F-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{00000011-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+                <c16:uniqueId val="{00000013-2E03-4E45-8C3C-EF6D9017B789}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-DB4A-4C4C-991C-1B1B262B3EB3}"/>
+              <c16:uniqueId val="{00000014-2E03-4E45-8C3C-EF6D9017B789}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-B1FA-42F5-84AC-FB2EB795E11C}"/>
+                <c16:uniqueId val="{00000001-9C40-4E57-8554-7ADD845FB129}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-B1FA-42F5-84AC-FB2EB795E11C}"/>
+                <c16:uniqueId val="{00000003-9C40-4E57-8554-7ADD845FB129}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-B1FA-42F5-84AC-FB2EB795E11C}"/>
+              <c16:uniqueId val="{00000004-9C40-4E57-8554-7ADD845FB129}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
0.6.3: writing checks that block packaging
Calibrated on accepted reports versus an unedited agent draft:
- process wording (cross-report, matched, not self-defined, attribute filter, narrative file)
- 'needs customer confirmation' at most twice per report
- hedging ('does not mean', 'cannot conclude', ...) at most max(5, 6 per 10,000 characters)
- 00 immediate issues and 03/04 top issues must name a resource or subscription; impact on all or none
- 00 conclusion must state amounts and name the most urgent resources
- build fingerprints the reports; package refuses reports edited by hand afterwards
Sample summary conclusion rewritten to pass.
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-yb_0tvu1\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-09jfy2fk\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE7CB789-C94B-4F32-AEED-2718A9E86021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D5C424-AF14-4533-B02D-5D7F4B5843EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17190" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="月度总览" sheetId="1" r:id="rId1"/>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-27T09:56:53.145316+00:00</t>
+    <t>2026-10-27T11:07:34.418527+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2C6F-4FAE-9EB0-C59B49A42ADE}"/>
+              <c16:uniqueId val="{00000000-3457-4E81-9BFD-345C9B0DA903}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-2C6F-4FAE-9EB0-C59B49A42ADE}"/>
+              <c16:uniqueId val="{00000001-3457-4E81-9BFD-345C9B0DA903}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C503-49C3-9E91-6C224CBF0505}"/>
+              <c16:uniqueId val="{00000000-003B-46F4-B6C4-C4C2F0C11223}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-C503-49C3-9E91-6C224CBF0505}"/>
+              <c16:uniqueId val="{00000001-003B-46F4-B6C4-C4C2F0C11223}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-C503-49C3-9E91-6C224CBF0505}"/>
+              <c16:uniqueId val="{00000002-003B-46F4-B6C4-C4C2F0C11223}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DA88-423D-BC40-4BE8BF19FCB0}"/>
+              <c16:uniqueId val="{00000000-892B-4954-9FEE-18BF2F404375}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-DA88-423D-BC40-4BE8BF19FCB0}"/>
+              <c16:uniqueId val="{00000001-892B-4954-9FEE-18BF2F404375}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{00000001-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{00000003-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{00000005-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{00000007-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{00000009-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{0000000B-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{0000000D-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{0000000F-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{00000011-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-2E03-4E45-8C3C-EF6D9017B789}"/>
+                <c16:uniqueId val="{00000013-B39C-4ABA-B8D9-E8F74823366A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-2E03-4E45-8C3C-EF6D9017B789}"/>
+              <c16:uniqueId val="{00000014-B39C-4ABA-B8D9-E8F74823366A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-9C40-4E57-8554-7ADD845FB129}"/>
+                <c16:uniqueId val="{00000001-222E-4B43-95DD-FA6384CE96EC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-9C40-4E57-8554-7ADD845FB129}"/>
+                <c16:uniqueId val="{00000003-222E-4B43-95DD-FA6384CE96EC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-9C40-4E57-8554-7ADD845FB129}"/>
+              <c16:uniqueId val="{00000004-222E-4B43-95DD-FA6384CE96EC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
0.6.4: fixes from a Claude Code offline run
- S-I8 (SSH password login with a public IP) now states the network result for port 22 instead of leaving it to the reader
- 00: default immediate issues no longer crash without a narrative; summary table shows the peer deviation count
- Markdown formatting no longer adds spaces around '=' (tags like key=value stay intact)
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-09jfy2fk\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-5yxkm8zf\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D5C424-AF14-4533-B02D-5D7F4B5843EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F49538-5D05-4D5D-80E1-0230AB7F2425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="月度总览" sheetId="1" r:id="rId1"/>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-27T11:07:34.418527+00:00</t>
+    <t>2026-10-27T13:22:17.643676+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3457-4E81-9BFD-345C9B0DA903}"/>
+              <c16:uniqueId val="{00000000-007C-47FC-A99D-0FBF4454EF5B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3457-4E81-9BFD-345C9B0DA903}"/>
+              <c16:uniqueId val="{00000001-007C-47FC-A99D-0FBF4454EF5B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-003B-46F4-B6C4-C4C2F0C11223}"/>
+              <c16:uniqueId val="{00000000-970D-4754-9EEC-3988779DEB96}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-003B-46F4-B6C4-C4C2F0C11223}"/>
+              <c16:uniqueId val="{00000001-970D-4754-9EEC-3988779DEB96}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-003B-46F4-B6C4-C4C2F0C11223}"/>
+              <c16:uniqueId val="{00000002-970D-4754-9EEC-3988779DEB96}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-892B-4954-9FEE-18BF2F404375}"/>
+              <c16:uniqueId val="{00000000-6CBD-42CD-8227-C439FCE341B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-892B-4954-9FEE-18BF2F404375}"/>
+              <c16:uniqueId val="{00000001-6CBD-42CD-8227-C439FCE341B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{00000001-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{00000003-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{00000005-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{00000007-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{00000009-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{0000000B-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{0000000D-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{0000000F-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{00000011-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-B39C-4ABA-B8D9-E8F74823366A}"/>
+                <c16:uniqueId val="{00000013-D52D-408B-A451-968906E92EF7}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-B39C-4ABA-B8D9-E8F74823366A}"/>
+              <c16:uniqueId val="{00000014-D52D-408B-A451-968906E92EF7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-222E-4B43-95DD-FA6384CE96EC}"/>
+                <c16:uniqueId val="{00000001-632A-4C8C-B4DE-9E27BF84CC73}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-222E-4B43-95DD-FA6384CE96EC}"/>
+                <c16:uniqueId val="{00000003-632A-4C8C-B4DE-9E27BF84CC73}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-222E-4B43-95DD-FA6384CE96EC}"/>
+              <c16:uniqueId val="{00000004-632A-4C8C-B4DE-9E27BF84CC73}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
0.6.5: action plans accept lists or '；'-separated strings
- 00/03/04 share one normalization: a narrative string is no longer split into one list item per character in 00; several items in 03/04 render as a sub-list instead of being joined
- quality-check fails on three or more consecutive one-character list items
- narrative-format.md: both forms documented for actionPlan
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-do642wo4\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-jluf97rf\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A6BD82-BC9E-4B96-8F67-21FDB21EFB24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6E0BEF-AD1A-4C38-B2BF-3F1D02FFA4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-29T15:39:31.447916+00:00</t>
+    <t>2026-10-29T15:57:22.064976+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D891-423F-A35E-E6FE9B69DC40}"/>
+              <c16:uniqueId val="{00000000-0A23-4011-91DA-497407C3DA81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D891-423F-A35E-E6FE9B69DC40}"/>
+              <c16:uniqueId val="{00000001-0A23-4011-91DA-497407C3DA81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F4EB-468D-8E1C-C2C6F1B9B181}"/>
+              <c16:uniqueId val="{00000000-3D27-479A-A455-1AA18D13F601}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-F4EB-468D-8E1C-C2C6F1B9B181}"/>
+              <c16:uniqueId val="{00000001-3D27-479A-A455-1AA18D13F601}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-F4EB-468D-8E1C-C2C6F1B9B181}"/>
+              <c16:uniqueId val="{00000002-3D27-479A-A455-1AA18D13F601}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7F46-4394-AEAE-A4404A4E14EE}"/>
+              <c16:uniqueId val="{00000000-5FCF-4854-87D4-57C5DB961339}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-7F46-4394-AEAE-A4404A4E14EE}"/>
+              <c16:uniqueId val="{00000001-5FCF-4854-87D4-57C5DB961339}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{00000001-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{00000003-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{00000005-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{00000007-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{00000009-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{0000000B-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{0000000D-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{0000000F-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{00000011-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-6284-4195-B9CD-523042B86863}"/>
+                <c16:uniqueId val="{00000013-665F-4B03-8975-492641CA1337}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-6284-4195-B9CD-523042B86863}"/>
+              <c16:uniqueId val="{00000014-665F-4B03-8975-492641CA1337}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-784C-49AB-A49E-0B52A1DDA608}"/>
+                <c16:uniqueId val="{00000001-F9FD-4F72-9D77-6DB0200C338B}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-784C-49AB-A49E-0B52A1DDA608}"/>
+                <c16:uniqueId val="{00000003-F9FD-4F72-9D77-6DB0200C338B}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-784C-49AB-A49E-0B52A1DDA608}"/>
+              <c16:uniqueId val="{00000004-F9FD-4F72-9D77-6DB0200C338B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
0.6.5: 02 summary tables; plain credential wording
- 02 Markdown: section 2 is four fixed summary tables (by subscription, by outcome, size changes, top 20 with node pools/VMSS on one row); the per-machine table is attached only up to report.vmDetailMaxRows machines (default 500), otherwise it stays in Excel
- 02 audit checks the summary numbers against the rows and the Excel subscription sheet
- quality-check fails on Markdown files over 500 KB
- S-I6: credential kinds in plain Chinese instead of API field names
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-jluf97rf\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-4z_oecii\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6E0BEF-AD1A-4C38-B2BF-3F1D02FFA4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACCEFFF-48CD-48B5-AAEB-85A0279E6AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="月度总览" sheetId="1" r:id="rId1"/>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-29T15:57:22.064976+00:00</t>
+    <t>2026-10-29T17:02:46.999275+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -1104,7 +1104,7 @@
     <t>10月费用预测（Azure Cost Management）</t>
   </si>
   <si>
-    <t>查询日期2026-10-29；已发生的日期为实际费用，其余为Azure预测值，不是账单金额。9月无费用的订阅预测接口不返回结果。</t>
+    <t>查询日期2026-10-30；已发生的日期为实际费用，其余为Azure预测值，不是账单金额。9月无费用的订阅预测接口不返回结果。</t>
   </si>
   <si>
     <t>10月截至查询日实际USD</t>
@@ -1779,7 +1779,7 @@
     <t>10月费用预测</t>
   </si>
   <si>
-    <t>查询日期2026-10-29；5个订阅有预测结果，其余0个订阅接口未返回预测；预测为Azure模型结果，不是账单</t>
+    <t>查询日期2026-10-30；5个订阅有预测结果，其余0个订阅接口未返回预测；预测为Azure模型结果，不是账单</t>
   </si>
   <si>
     <t>费用变化原因</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0A23-4011-91DA-497407C3DA81}"/>
+              <c16:uniqueId val="{00000000-D45B-4E7D-9811-F01274454B7A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-0A23-4011-91DA-497407C3DA81}"/>
+              <c16:uniqueId val="{00000001-D45B-4E7D-9811-F01274454B7A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3D27-479A-A455-1AA18D13F601}"/>
+              <c16:uniqueId val="{00000000-4F06-42EC-BE12-E9093014F3B5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3D27-479A-A455-1AA18D13F601}"/>
+              <c16:uniqueId val="{00000001-4F06-42EC-BE12-E9093014F3B5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3D27-479A-A455-1AA18D13F601}"/>
+              <c16:uniqueId val="{00000002-4F06-42EC-BE12-E9093014F3B5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5FCF-4854-87D4-57C5DB961339}"/>
+              <c16:uniqueId val="{00000000-C2D2-4485-BE61-6B50674C4D95}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5FCF-4854-87D4-57C5DB961339}"/>
+              <c16:uniqueId val="{00000001-C2D2-4485-BE61-6B50674C4D95}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{00000001-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{00000003-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{00000005-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{00000007-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{00000009-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{0000000B-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{0000000D-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{0000000F-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{00000011-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-665F-4B03-8975-492641CA1337}"/>
+                <c16:uniqueId val="{00000013-6F70-4313-B4FA-491B36A13618}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-665F-4B03-8975-492641CA1337}"/>
+              <c16:uniqueId val="{00000014-6F70-4313-B4FA-491B36A13618}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-F9FD-4F72-9D77-6DB0200C338B}"/>
+                <c16:uniqueId val="{00000001-9B7D-4670-A00A-6E0ECC9F71B0}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-F9FD-4F72-9D77-6DB0200C338B}"/>
+                <c16:uniqueId val="{00000003-9B7D-4670-A00A-6E0ECC9F71B0}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-F9FD-4F72-9D77-6DB0200C338B}"/>
+              <c16:uniqueId val="{00000004-9B7D-4670-A00A-6E0ECC9F71B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
0.6.6: version end of support and retirement checks (R9)
- Service Health retirement notices with impacted resources (Advisor join as fallback), deduplicated against Advisor retirement recommendations
- MySQL/PostgreSQL engine versions (paid extended support stated), Azure Cache for Redis versions and tier retirement
- VM and scale set operating systems (CentOS, Ubuntu, RHEL, Windows Server, Rocky, AlmaLinux, Debian, SLES) from instanceView or image reference
- App Service stack versions from Resource Graph, else one config/web GET per site keeping version fields only
- Application Gateway certificate expiry from the public certificate data (new dependency: cryptography)
- Support dates in vendor/lifecycle/lifecycle.json with a source per entry; a reminder when not reviewed for 180 days
- Severity: passed -> high, within 180 days -> medium, within 365 days -> low; resources grouped per subscription; items that could not be judged are counted under scope and limits
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-4z_oecii\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-gq0eyj71\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACCEFFF-48CD-48B5-AAEB-85A0279E6AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DE099B5-AB77-448F-BF72-492477F01F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2280" yWindow="2280" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-29T17:02:46.999275+00:00</t>
+    <t>2026-10-29T18:20:54.376824+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D45B-4E7D-9811-F01274454B7A}"/>
+              <c16:uniqueId val="{00000000-CD0A-4D88-B8C3-17FAE29FD5C7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D45B-4E7D-9811-F01274454B7A}"/>
+              <c16:uniqueId val="{00000001-CD0A-4D88-B8C3-17FAE29FD5C7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4F06-42EC-BE12-E9093014F3B5}"/>
+              <c16:uniqueId val="{00000000-DD54-4197-BEE6-FDD0C113B966}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4F06-42EC-BE12-E9093014F3B5}"/>
+              <c16:uniqueId val="{00000001-DD54-4197-BEE6-FDD0C113B966}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4F06-42EC-BE12-E9093014F3B5}"/>
+              <c16:uniqueId val="{00000002-DD54-4197-BEE6-FDD0C113B966}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C2D2-4485-BE61-6B50674C4D95}"/>
+              <c16:uniqueId val="{00000000-845C-4C60-AE8F-EFFEB870872C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-C2D2-4485-BE61-6B50674C4D95}"/>
+              <c16:uniqueId val="{00000001-845C-4C60-AE8F-EFFEB870872C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{00000001-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{00000003-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{00000005-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{00000007-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{00000009-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{0000000B-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{0000000D-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{0000000F-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{00000011-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-6F70-4313-B4FA-491B36A13618}"/>
+                <c16:uniqueId val="{00000013-C6D3-4861-81ED-0470CB27AB8A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-6F70-4313-B4FA-491B36A13618}"/>
+              <c16:uniqueId val="{00000014-C6D3-4861-81ED-0470CB27AB8A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-9B7D-4670-A00A-6E0ECC9F71B0}"/>
+                <c16:uniqueId val="{00000001-2D80-4B5F-B85A-67EFFC6519DF}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-9B7D-4670-A00A-6E0ECC9F71B0}"/>
+                <c16:uniqueId val="{00000003-2D80-4B5F-B85A-67EFFC6519DF}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-9B7D-4670-A00A-6E0ECC9F71B0}"/>
+              <c16:uniqueId val="{00000004-2D80-4B5F-B85A-67EFFC6519DF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
0.7.0: resumable cost collection; smaller cost model
- collect --part cost --resume reuses reads of the same month and query that succeeded within 7 days (cost, supplement and RI/SP queries per subscription; database/storage/log, orphan and VM usage steps as a whole); failed or denied reads are repeated
- per-resource costs of subscriptions with more than 100 resource groups are read in batches of 50 resource groups; cost outside resource groups is added as one row so the total is unchanged
- RI/SP: totals by pricing model from a small per-subscription query; per-resource pricing only for virtual machines and scale sets (falls back to local filtering if the type filter is refused); report numbers unchanged
- findings/cost/model.json keeps totals and the top 20 resources; every per-resource row moves to findings/cost/resources.json (compact); older model files still read
- an interrupted collection prints the --resume command; equal-cost resources sorted deterministically
</commit_message>
<xml_diff>
--- a/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
+++ b/examples/sample-output/Contoso_Azure巡检报告_2026年10月/01_9月月度成本巡检报告.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-gq0eyj71\2026-09\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wez\AppData\Local\Temp\azinspect-sample-9n18lti6\2026-09\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DE099B5-AB77-448F-BF72-492477F01F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE65942-75F1-42C1-96EA-153F6F2AFF93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2280" yWindow="2280" windowWidth="16920" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -174,7 +174,7 @@
     <t>数据查询时间</t>
   </si>
   <si>
-    <t>2026-10-29T18:20:54.376824+00:00</t>
+    <t>2026-10-29T21:12:04.445154+00:00</t>
   </si>
   <si>
     <t>完整月份费用按查询时结果列示</t>
@@ -894,18 +894,18 @@
     <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a4/resourcegroups/data-rg/providers/microsoft.cognitiveservices/accounts/data-openai</t>
   </si>
   <si>
+    <t>pay-mysql-prod</t>
+  </si>
+  <si>
+    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.dbformysql/flexibleservers/pay-mysql-prod</t>
+  </si>
+  <si>
     <t>shop-mysql-prod</t>
   </si>
   <si>
     <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a1/resourcegroups/shop-rg/providers/microsoft.dbformysql/flexibleservers/shop-mysql-prod</t>
   </si>
   <si>
-    <t>pay-mysql-prod</t>
-  </si>
-  <si>
-    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.dbformysql/flexibleservers/pay-mysql-prod</t>
-  </si>
-  <si>
     <t>pay-pg-prod</t>
   </si>
   <si>
@@ -948,6 +948,18 @@
     <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a5/resourcegroups/network-rg/providers/microsoft.network/virtualnetworkgateways/shared-vpn</t>
   </si>
   <si>
+    <t>pay-api-01</t>
+  </si>
+  <si>
+    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/virtualmachines/pay-api-01</t>
+  </si>
+  <si>
+    <t>pay-api-02</t>
+  </si>
+  <si>
+    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/virtualmachines/pay-api-02</t>
+  </si>
+  <si>
     <t>shop-web-01</t>
   </si>
   <si>
@@ -978,18 +990,6 @@
     <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a2/resourcegroups/shop-test-rg/providers/microsoft.compute/virtualmachines/shop-web-test-01</t>
   </si>
   <si>
-    <t>pay-api-01</t>
-  </si>
-  <si>
-    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/virtualmachines/pay-api-01</t>
-  </si>
-  <si>
-    <t>pay-api-02</t>
-  </si>
-  <si>
-    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/virtualmachines/pay-api-02</t>
-  </si>
-  <si>
     <t>data-worker-01</t>
   </si>
   <si>
@@ -1020,6 +1020,24 @@
     <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.keyvault/vaults/pay-kv</t>
   </si>
   <si>
+    <t>data-etl-01-osdisk</t>
+  </si>
+  <si>
+    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a4/resourcegroups/data-rg/providers/microsoft.compute/disks/data-etl-01-osdisk</t>
+  </si>
+  <si>
+    <t>pay-api-01-osdisk</t>
+  </si>
+  <si>
+    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/disks/pay-api-01-osdisk</t>
+  </si>
+  <si>
+    <t>pay-api-02-osdisk</t>
+  </si>
+  <si>
+    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/disks/pay-api-02-osdisk</t>
+  </si>
+  <si>
     <t>shop-batch-01-osdisk</t>
   </si>
   <si>
@@ -1060,24 +1078,6 @@
   </si>
   <si>
     <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a2/resourcegroups/shop-test-rg/providers/microsoft.compute/disks/shop-web-test-01-osdisk</t>
-  </si>
-  <si>
-    <t>pay-api-01-osdisk</t>
-  </si>
-  <si>
-    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/disks/pay-api-01-osdisk</t>
-  </si>
-  <si>
-    <t>pay-api-02-osdisk</t>
-  </si>
-  <si>
-    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a3/resourcegroups/pay-rg/providers/microsoft.compute/disks/pay-api-02-osdisk</t>
-  </si>
-  <si>
-    <t>data-etl-01-osdisk</t>
-  </si>
-  <si>
-    <t>/subscriptions/5a1e0c01-1111-4c2a-9a10-0000000000a4/resourcegroups/data-rg/providers/microsoft.compute/disks/data-etl-01-osdisk</t>
   </si>
   <si>
     <t>payreceipts</t>
@@ -2299,7 +2299,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-CD0A-4D88-B8C3-17FAE29FD5C7}"/>
+              <c16:uniqueId val="{00000000-3E38-4F31-B00B-BDBE5934EEC3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-CD0A-4D88-B8C3-17FAE29FD5C7}"/>
+              <c16:uniqueId val="{00000001-3E38-4F31-B00B-BDBE5934EEC3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2919,7 +2919,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DD54-4197-BEE6-FDD0C113B966}"/>
+              <c16:uniqueId val="{00000000-2141-41D1-8994-89464ED33A2F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3076,7 +3076,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-DD54-4197-BEE6-FDD0C113B966}"/>
+              <c16:uniqueId val="{00000001-2141-41D1-8994-89464ED33A2F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3311,7 +3311,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-DD54-4197-BEE6-FDD0C113B966}"/>
+              <c16:uniqueId val="{00000002-2141-41D1-8994-89464ED33A2F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3478,7 +3478,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-845C-4C60-AE8F-EFFEB870872C}"/>
+              <c16:uniqueId val="{00000000-E285-47A6-9515-54C3DDFBC9A6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3566,7 +3566,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-845C-4C60-AE8F-EFFEB870872C}"/>
+              <c16:uniqueId val="{00000001-E285-47A6-9515-54C3DDFBC9A6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3690,7 +3690,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{00000001-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3711,7 +3711,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{00000003-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3732,7 +3732,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{00000005-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3753,7 +3753,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{00000007-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3763,7 +3763,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{00000009-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3773,7 +3773,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{0000000B-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3783,7 +3783,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000D-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{0000000D-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3793,7 +3793,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000F-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{0000000F-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3803,7 +3803,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000011-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{00000011-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3813,7 +3813,7 @@
             <c:bubble3D val="0"/>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000013-C6D3-4861-81ED-0470CB27AB8A}"/>
+                <c16:uniqueId val="{00000013-4A57-4213-997D-1FEF5F5EFEC4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -3896,7 +3896,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000014-C6D3-4861-81ED-0470CB27AB8A}"/>
+              <c16:uniqueId val="{00000014-4A57-4213-997D-1FEF5F5EFEC4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4016,7 +4016,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-2D80-4B5F-B85A-67EFFC6519DF}"/>
+                <c16:uniqueId val="{00000001-A27C-463C-934F-C00A806942C6}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4037,7 +4037,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-2D80-4B5F-B85A-67EFFC6519DF}"/>
+                <c16:uniqueId val="{00000003-A27C-463C-934F-C00A806942C6}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -4072,7 +4072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-2D80-4B5F-B85A-67EFFC6519DF}"/>
+              <c16:uniqueId val="{00000004-A27C-463C-934F-C00A806942C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5068,10 +5068,10 @@
     </row>
     <row r="9" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>264</v>
@@ -5088,10 +5088,10 @@
     </row>
     <row r="10" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>266</v>
@@ -5268,10 +5268,10 @@
     </row>
     <row r="19" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>282</v>
@@ -5288,10 +5288,10 @@
     </row>
     <row r="20" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>284</v>
@@ -5348,10 +5348,10 @@
     </row>
     <row r="23" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>290</v>
@@ -5368,10 +5368,10 @@
     </row>
     <row r="24" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>292</v>
@@ -5388,10 +5388,10 @@
     </row>
     <row r="25" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>294</v>
@@ -5506,12 +5506,12 @@
         <v>305</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" ht="75" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>306</v>
@@ -5526,12 +5526,12 @@
         <v>307</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="75" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>308</v>
@@ -5546,12 +5546,12 @@
         <v>309</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" ht="75" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>310</v>
@@ -5628,10 +5628,10 @@
     </row>
     <row r="37" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>318</v>
@@ -5646,12 +5646,12 @@
         <v>319</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="75" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>320</v>
@@ -5666,12 +5666,12 @@
         <v>321</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="75" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>322</v>
@@ -5686,12 +5686,12 @@
         <v>323</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="75" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" ht="87.5" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>324</v>
@@ -7411,7 +7411,7 @@
         <v>246</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>466</v>
@@ -7450,7 +7450,7 @@
         <v>247</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>466</v>

</xml_diff>